<commit_message>
Remove temporary Excel file and update main Excel file with new data
</commit_message>
<xml_diff>
--- a/public/xlsx/736067c4-bd56-4c2e-8e0e-6bd9cfa9f39c.xlsx
+++ b/public/xlsx/736067c4-bd56-4c2e-8e0e-6bd9cfa9f39c.xlsx
@@ -97,11 +97,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$R$ -416]#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="dd/MM/yyyy"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -150,11 +149,6 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -182,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="13">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -197,9 +191,7 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -207,21 +199,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -446,12 +428,12 @@
     <col customWidth="1" min="5" max="5" width="17.75"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" ht="30.0" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1">
+    <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -498,8 +480,8 @@
       <c r="B6" s="9"/>
       <c r="C6" s="10"/>
       <c r="D6" s="9"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="12">
+      <c r="E6" s="9"/>
+      <c r="F6" s="11">
         <f>IFERROR(VLOOKUP(E6, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -509,10 +491,10 @@
         <v>2.0</v>
       </c>
       <c r="B7" s="9"/>
-      <c r="C7" s="13"/>
+      <c r="C7" s="10"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
-      <c r="F7" s="12">
+      <c r="F7" s="11">
         <f>IFERROR(VLOOKUP(E7, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -525,7 +507,7 @@
       <c r="C8" s="10"/>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
-      <c r="F8" s="12">
+      <c r="F8" s="11">
         <f>IFERROR(VLOOKUP(E8, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -538,7 +520,7 @@
       <c r="C9" s="10"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
-      <c r="F9" s="12">
+      <c r="F9" s="11">
         <f>IFERROR(VLOOKUP(E9, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -551,7 +533,7 @@
       <c r="C10" s="10"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
-      <c r="F10" s="12">
+      <c r="F10" s="11">
         <f>IFERROR(VLOOKUP(E10, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -564,7 +546,7 @@
       <c r="C11" s="10"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
-      <c r="F11" s="12">
+      <c r="F11" s="11">
         <f>IFERROR(VLOOKUP(E11, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -577,7 +559,7 @@
       <c r="C12" s="10"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
-      <c r="F12" s="12">
+      <c r="F12" s="11">
         <f>IFERROR(VLOOKUP(E12, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -590,7 +572,7 @@
       <c r="C13" s="10"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
-      <c r="F13" s="12">
+      <c r="F13" s="11">
         <f>IFERROR(VLOOKUP(E13, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -603,7 +585,7 @@
       <c r="C14" s="10"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
-      <c r="F14" s="12">
+      <c r="F14" s="11">
         <f>IFERROR(VLOOKUP(E14, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -616,7 +598,7 @@
       <c r="C15" s="10"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
-      <c r="F15" s="12">
+      <c r="F15" s="11">
         <f>IFERROR(VLOOKUP(E15, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -629,7 +611,7 @@
       <c r="C16" s="10"/>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
-      <c r="F16" s="12">
+      <c r="F16" s="11">
         <f>IFERROR(VLOOKUP(E16, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -642,7 +624,7 @@
       <c r="C17" s="10"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
-      <c r="F17" s="12">
+      <c r="F17" s="11">
         <f>IFERROR(VLOOKUP(E17, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -655,7 +637,7 @@
       <c r="C18" s="10"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
-      <c r="F18" s="12">
+      <c r="F18" s="11">
         <f>IFERROR(VLOOKUP(E18, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -668,7 +650,7 @@
       <c r="C19" s="10"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
-      <c r="F19" s="12">
+      <c r="F19" s="11">
         <f>IFERROR(VLOOKUP(E19, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -681,7 +663,7 @@
       <c r="C20" s="10"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
-      <c r="F20" s="12">
+      <c r="F20" s="11">
         <f>IFERROR(VLOOKUP(E20, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -694,7 +676,7 @@
       <c r="C21" s="10"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
-      <c r="F21" s="12">
+      <c r="F21" s="11">
         <f>IFERROR(VLOOKUP(E21, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -707,7 +689,7 @@
       <c r="C22" s="10"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
-      <c r="F22" s="12">
+      <c r="F22" s="11">
         <f>IFERROR(VLOOKUP(E22, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -720,7 +702,7 @@
       <c r="C23" s="10"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
-      <c r="F23" s="12">
+      <c r="F23" s="11">
         <f>IFERROR(VLOOKUP(E23, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -733,7 +715,7 @@
       <c r="C24" s="10"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
-      <c r="F24" s="12">
+      <c r="F24" s="11">
         <f>IFERROR(VLOOKUP(E24, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -746,7 +728,7 @@
       <c r="C25" s="10"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
-      <c r="F25" s="12">
+      <c r="F25" s="11">
         <f>IFERROR(VLOOKUP(E25, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -759,7 +741,7 @@
       <c r="C26" s="10"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
-      <c r="F26" s="12">
+      <c r="F26" s="11">
         <f>IFERROR(VLOOKUP(E26, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -772,7 +754,7 @@
       <c r="C27" s="10"/>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
-      <c r="F27" s="12">
+      <c r="F27" s="11">
         <f>IFERROR(VLOOKUP(E27, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -785,7 +767,7 @@
       <c r="C28" s="10"/>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
-      <c r="F28" s="12">
+      <c r="F28" s="11">
         <f>IFERROR(VLOOKUP(E28, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -798,7 +780,7 @@
       <c r="C29" s="10"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
-      <c r="F29" s="12">
+      <c r="F29" s="11">
         <f>IFERROR(VLOOKUP(E29, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -811,7 +793,7 @@
       <c r="C30" s="10"/>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
-      <c r="F30" s="12">
+      <c r="F30" s="11">
         <f>IFERROR(VLOOKUP(E30, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -824,7 +806,7 @@
       <c r="C31" s="10"/>
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
-      <c r="F31" s="12">
+      <c r="F31" s="11">
         <f>IFERROR(VLOOKUP(E31, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -837,7 +819,7 @@
       <c r="C32" s="10"/>
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
-      <c r="F32" s="12">
+      <c r="F32" s="11">
         <f>IFERROR(VLOOKUP(E32, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -850,7 +832,7 @@
       <c r="C33" s="10"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
-      <c r="F33" s="12">
+      <c r="F33" s="11">
         <f>IFERROR(VLOOKUP(E33, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -863,7 +845,7 @@
       <c r="C34" s="10"/>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
-      <c r="F34" s="12">
+      <c r="F34" s="11">
         <f>IFERROR(VLOOKUP(E34, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -876,7 +858,7 @@
       <c r="C35" s="10"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
-      <c r="F35" s="12">
+      <c r="F35" s="11">
         <f>IFERROR(VLOOKUP(E35, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -889,7 +871,7 @@
       <c r="C36" s="10"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
-      <c r="F36" s="12">
+      <c r="F36" s="11">
         <f>IFERROR(VLOOKUP(E36, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -902,7 +884,7 @@
       <c r="C37" s="10"/>
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
-      <c r="F37" s="12">
+      <c r="F37" s="11">
         <f>IFERROR(VLOOKUP(E37, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -915,7 +897,7 @@
       <c r="C38" s="10"/>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
-      <c r="F38" s="12">
+      <c r="F38" s="11">
         <f>IFERROR(VLOOKUP(E38, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -928,7 +910,7 @@
       <c r="C39" s="10"/>
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
-      <c r="F39" s="12">
+      <c r="F39" s="11">
         <f>IFERROR(VLOOKUP(E39, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -941,7 +923,7 @@
       <c r="C40" s="10"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
-      <c r="F40" s="12">
+      <c r="F40" s="11">
         <f>IFERROR(VLOOKUP(E40, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -954,7 +936,7 @@
       <c r="C41" s="10"/>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
-      <c r="F41" s="12">
+      <c r="F41" s="11">
         <f>IFERROR(VLOOKUP(E41, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -967,7 +949,7 @@
       <c r="C42" s="10"/>
       <c r="D42" s="9"/>
       <c r="E42" s="9"/>
-      <c r="F42" s="12">
+      <c r="F42" s="11">
         <f>IFERROR(VLOOKUP(E42, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -980,7 +962,7 @@
       <c r="C43" s="10"/>
       <c r="D43" s="9"/>
       <c r="E43" s="9"/>
-      <c r="F43" s="12">
+      <c r="F43" s="11">
         <f>IFERROR(VLOOKUP(E43, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -993,7 +975,7 @@
       <c r="C44" s="10"/>
       <c r="D44" s="9"/>
       <c r="E44" s="9"/>
-      <c r="F44" s="12">
+      <c r="F44" s="11">
         <f>IFERROR(VLOOKUP(E44, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1006,7 +988,7 @@
       <c r="C45" s="10"/>
       <c r="D45" s="9"/>
       <c r="E45" s="9"/>
-      <c r="F45" s="12">
+      <c r="F45" s="11">
         <f>IFERROR(VLOOKUP(E45, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1019,7 +1001,7 @@
       <c r="C46" s="10"/>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
-      <c r="F46" s="12">
+      <c r="F46" s="11">
         <f>IFERROR(VLOOKUP(E46, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1032,7 +1014,7 @@
       <c r="C47" s="10"/>
       <c r="D47" s="9"/>
       <c r="E47" s="9"/>
-      <c r="F47" s="12">
+      <c r="F47" s="11">
         <f>IFERROR(VLOOKUP(E47, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1045,7 +1027,7 @@
       <c r="C48" s="10"/>
       <c r="D48" s="9"/>
       <c r="E48" s="9"/>
-      <c r="F48" s="12">
+      <c r="F48" s="11">
         <f>IFERROR(VLOOKUP(E48, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1058,7 +1040,7 @@
       <c r="C49" s="10"/>
       <c r="D49" s="9"/>
       <c r="E49" s="9"/>
-      <c r="F49" s="12">
+      <c r="F49" s="11">
         <f>IFERROR(VLOOKUP(E49, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1071,7 +1053,7 @@
       <c r="C50" s="10"/>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
-      <c r="F50" s="12">
+      <c r="F50" s="11">
         <f>IFERROR(VLOOKUP(E50, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1084,7 +1066,7 @@
       <c r="C51" s="10"/>
       <c r="D51" s="9"/>
       <c r="E51" s="9"/>
-      <c r="F51" s="12">
+      <c r="F51" s="11">
         <f>IFERROR(VLOOKUP(E51, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1097,7 +1079,7 @@
       <c r="C52" s="10"/>
       <c r="D52" s="9"/>
       <c r="E52" s="9"/>
-      <c r="F52" s="12">
+      <c r="F52" s="11">
         <f>IFERROR(VLOOKUP(E52, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1110,7 +1092,7 @@
       <c r="C53" s="10"/>
       <c r="D53" s="9"/>
       <c r="E53" s="9"/>
-      <c r="F53" s="12">
+      <c r="F53" s="11">
         <f>IFERROR(VLOOKUP(E53, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1123,7 +1105,7 @@
       <c r="C54" s="10"/>
       <c r="D54" s="9"/>
       <c r="E54" s="9"/>
-      <c r="F54" s="12">
+      <c r="F54" s="11">
         <f>IFERROR(VLOOKUP(E54, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1136,7 +1118,7 @@
       <c r="C55" s="10"/>
       <c r="D55" s="9"/>
       <c r="E55" s="9"/>
-      <c r="F55" s="12">
+      <c r="F55" s="11">
         <f>IFERROR(VLOOKUP(E55, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1149,7 +1131,7 @@
       <c r="C56" s="10"/>
       <c r="D56" s="9"/>
       <c r="E56" s="9"/>
-      <c r="F56" s="12">
+      <c r="F56" s="11">
         <f>IFERROR(VLOOKUP(E56, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1162,7 +1144,7 @@
       <c r="C57" s="10"/>
       <c r="D57" s="9"/>
       <c r="E57" s="9"/>
-      <c r="F57" s="12">
+      <c r="F57" s="11">
         <f>IFERROR(VLOOKUP(E57, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1175,7 +1157,7 @@
       <c r="C58" s="10"/>
       <c r="D58" s="9"/>
       <c r="E58" s="9"/>
-      <c r="F58" s="12">
+      <c r="F58" s="11">
         <f>IFERROR(VLOOKUP(E58, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1188,7 +1170,7 @@
       <c r="C59" s="10"/>
       <c r="D59" s="9"/>
       <c r="E59" s="9"/>
-      <c r="F59" s="12">
+      <c r="F59" s="11">
         <f>IFERROR(VLOOKUP(E59, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1201,7 +1183,7 @@
       <c r="C60" s="10"/>
       <c r="D60" s="9"/>
       <c r="E60" s="9"/>
-      <c r="F60" s="12">
+      <c r="F60" s="11">
         <f>IFERROR(VLOOKUP(E60, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1214,7 +1196,7 @@
       <c r="C61" s="10"/>
       <c r="D61" s="9"/>
       <c r="E61" s="9"/>
-      <c r="F61" s="12">
+      <c r="F61" s="11">
         <f>IFERROR(VLOOKUP(E61, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1227,7 +1209,7 @@
       <c r="C62" s="10"/>
       <c r="D62" s="9"/>
       <c r="E62" s="9"/>
-      <c r="F62" s="12">
+      <c r="F62" s="11">
         <f>IFERROR(VLOOKUP(E62, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1240,7 +1222,7 @@
       <c r="C63" s="10"/>
       <c r="D63" s="9"/>
       <c r="E63" s="9"/>
-      <c r="F63" s="12">
+      <c r="F63" s="11">
         <f>IFERROR(VLOOKUP(E63, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1253,7 +1235,7 @@
       <c r="C64" s="10"/>
       <c r="D64" s="9"/>
       <c r="E64" s="9"/>
-      <c r="F64" s="12">
+      <c r="F64" s="11">
         <f>IFERROR(VLOOKUP(E64, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1266,7 +1248,7 @@
       <c r="C65" s="10"/>
       <c r="D65" s="9"/>
       <c r="E65" s="9"/>
-      <c r="F65" s="12">
+      <c r="F65" s="11">
         <f>IFERROR(VLOOKUP(E65, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1279,7 +1261,7 @@
       <c r="C66" s="10"/>
       <c r="D66" s="9"/>
       <c r="E66" s="9"/>
-      <c r="F66" s="12">
+      <c r="F66" s="11">
         <f>IFERROR(VLOOKUP(E66, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1292,7 +1274,7 @@
       <c r="C67" s="10"/>
       <c r="D67" s="9"/>
       <c r="E67" s="9"/>
-      <c r="F67" s="12">
+      <c r="F67" s="11">
         <f>IFERROR(VLOOKUP(E67, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1305,7 +1287,7 @@
       <c r="C68" s="10"/>
       <c r="D68" s="9"/>
       <c r="E68" s="9"/>
-      <c r="F68" s="12">
+      <c r="F68" s="11">
         <f>IFERROR(VLOOKUP(E68, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1318,7 +1300,7 @@
       <c r="C69" s="10"/>
       <c r="D69" s="9"/>
       <c r="E69" s="9"/>
-      <c r="F69" s="12">
+      <c r="F69" s="11">
         <f>IFERROR(VLOOKUP(E69, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1331,7 +1313,7 @@
       <c r="C70" s="10"/>
       <c r="D70" s="9"/>
       <c r="E70" s="9"/>
-      <c r="F70" s="12">
+      <c r="F70" s="11">
         <f>IFERROR(VLOOKUP(E70, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1344,7 +1326,7 @@
       <c r="C71" s="10"/>
       <c r="D71" s="9"/>
       <c r="E71" s="9"/>
-      <c r="F71" s="12">
+      <c r="F71" s="11">
         <f>IFERROR(VLOOKUP(E71, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1357,7 +1339,7 @@
       <c r="C72" s="10"/>
       <c r="D72" s="9"/>
       <c r="E72" s="9"/>
-      <c r="F72" s="12">
+      <c r="F72" s="11">
         <f>IFERROR(VLOOKUP(E72, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1370,7 +1352,7 @@
       <c r="C73" s="10"/>
       <c r="D73" s="9"/>
       <c r="E73" s="9"/>
-      <c r="F73" s="12">
+      <c r="F73" s="11">
         <f>IFERROR(VLOOKUP(E73, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1383,7 +1365,7 @@
       <c r="C74" s="10"/>
       <c r="D74" s="9"/>
       <c r="E74" s="9"/>
-      <c r="F74" s="12">
+      <c r="F74" s="11">
         <f>IFERROR(VLOOKUP(E74, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1396,7 +1378,7 @@
       <c r="C75" s="10"/>
       <c r="D75" s="9"/>
       <c r="E75" s="9"/>
-      <c r="F75" s="12">
+      <c r="F75" s="11">
         <f>IFERROR(VLOOKUP(E75, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1409,7 +1391,7 @@
       <c r="C76" s="10"/>
       <c r="D76" s="9"/>
       <c r="E76" s="9"/>
-      <c r="F76" s="12">
+      <c r="F76" s="11">
         <f>IFERROR(VLOOKUP(E76, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1422,7 +1404,7 @@
       <c r="C77" s="10"/>
       <c r="D77" s="9"/>
       <c r="E77" s="9"/>
-      <c r="F77" s="12">
+      <c r="F77" s="11">
         <f>IFERROR(VLOOKUP(E77, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1435,7 +1417,7 @@
       <c r="C78" s="10"/>
       <c r="D78" s="9"/>
       <c r="E78" s="9"/>
-      <c r="F78" s="12">
+      <c r="F78" s="11">
         <f>IFERROR(VLOOKUP(E78, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1448,7 +1430,7 @@
       <c r="C79" s="10"/>
       <c r="D79" s="9"/>
       <c r="E79" s="9"/>
-      <c r="F79" s="12">
+      <c r="F79" s="11">
         <f>IFERROR(VLOOKUP(E79, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1461,7 +1443,7 @@
       <c r="C80" s="10"/>
       <c r="D80" s="9"/>
       <c r="E80" s="9"/>
-      <c r="F80" s="12">
+      <c r="F80" s="11">
         <f>IFERROR(VLOOKUP(E80, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1474,7 +1456,7 @@
       <c r="C81" s="10"/>
       <c r="D81" s="9"/>
       <c r="E81" s="9"/>
-      <c r="F81" s="12">
+      <c r="F81" s="11">
         <f>IFERROR(VLOOKUP(E81, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1487,7 +1469,7 @@
       <c r="C82" s="10"/>
       <c r="D82" s="9"/>
       <c r="E82" s="9"/>
-      <c r="F82" s="12">
+      <c r="F82" s="11">
         <f>IFERROR(VLOOKUP(E82, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1500,7 +1482,7 @@
       <c r="C83" s="10"/>
       <c r="D83" s="9"/>
       <c r="E83" s="9"/>
-      <c r="F83" s="12">
+      <c r="F83" s="11">
         <f>IFERROR(VLOOKUP(E83, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1513,7 +1495,7 @@
       <c r="C84" s="10"/>
       <c r="D84" s="9"/>
       <c r="E84" s="9"/>
-      <c r="F84" s="12">
+      <c r="F84" s="11">
         <f>IFERROR(VLOOKUP(E84, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1526,7 +1508,7 @@
       <c r="C85" s="10"/>
       <c r="D85" s="9"/>
       <c r="E85" s="9"/>
-      <c r="F85" s="12">
+      <c r="F85" s="11">
         <f>IFERROR(VLOOKUP(E85, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1539,7 +1521,7 @@
       <c r="C86" s="10"/>
       <c r="D86" s="9"/>
       <c r="E86" s="9"/>
-      <c r="F86" s="12">
+      <c r="F86" s="11">
         <f>IFERROR(VLOOKUP(E86, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1552,7 +1534,7 @@
       <c r="C87" s="10"/>
       <c r="D87" s="9"/>
       <c r="E87" s="9"/>
-      <c r="F87" s="12">
+      <c r="F87" s="11">
         <f>IFERROR(VLOOKUP(E87, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1565,7 +1547,7 @@
       <c r="C88" s="10"/>
       <c r="D88" s="9"/>
       <c r="E88" s="9"/>
-      <c r="F88" s="12">
+      <c r="F88" s="11">
         <f>IFERROR(VLOOKUP(E88, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1578,7 +1560,7 @@
       <c r="C89" s="10"/>
       <c r="D89" s="9"/>
       <c r="E89" s="9"/>
-      <c r="F89" s="12">
+      <c r="F89" s="11">
         <f>IFERROR(VLOOKUP(E89, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1591,7 +1573,7 @@
       <c r="C90" s="10"/>
       <c r="D90" s="9"/>
       <c r="E90" s="9"/>
-      <c r="F90" s="12">
+      <c r="F90" s="11">
         <f>IFERROR(VLOOKUP(E90, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1604,7 +1586,7 @@
       <c r="C91" s="10"/>
       <c r="D91" s="9"/>
       <c r="E91" s="9"/>
-      <c r="F91" s="12">
+      <c r="F91" s="11">
         <f>IFERROR(VLOOKUP(E91, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1617,7 +1599,7 @@
       <c r="C92" s="10"/>
       <c r="D92" s="9"/>
       <c r="E92" s="9"/>
-      <c r="F92" s="12">
+      <c r="F92" s="11">
         <f>IFERROR(VLOOKUP(E92, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1630,7 +1612,7 @@
       <c r="C93" s="10"/>
       <c r="D93" s="9"/>
       <c r="E93" s="9"/>
-      <c r="F93" s="12">
+      <c r="F93" s="11">
         <f>IFERROR(VLOOKUP(E93, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1643,7 +1625,7 @@
       <c r="C94" s="10"/>
       <c r="D94" s="9"/>
       <c r="E94" s="9"/>
-      <c r="F94" s="12">
+      <c r="F94" s="11">
         <f>IFERROR(VLOOKUP(E94, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1656,7 +1638,7 @@
       <c r="C95" s="10"/>
       <c r="D95" s="9"/>
       <c r="E95" s="9"/>
-      <c r="F95" s="12">
+      <c r="F95" s="11">
         <f>IFERROR(VLOOKUP(E95, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1669,7 +1651,7 @@
       <c r="C96" s="10"/>
       <c r="D96" s="9"/>
       <c r="E96" s="9"/>
-      <c r="F96" s="12">
+      <c r="F96" s="11">
         <f>IFERROR(VLOOKUP(E96, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1682,7 +1664,7 @@
       <c r="C97" s="10"/>
       <c r="D97" s="9"/>
       <c r="E97" s="9"/>
-      <c r="F97" s="12">
+      <c r="F97" s="11">
         <f>IFERROR(VLOOKUP(E97, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1695,7 +1677,7 @@
       <c r="C98" s="10"/>
       <c r="D98" s="9"/>
       <c r="E98" s="9"/>
-      <c r="F98" s="12">
+      <c r="F98" s="11">
         <f>IFERROR(VLOOKUP(E98, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1708,7 +1690,7 @@
       <c r="C99" s="10"/>
       <c r="D99" s="9"/>
       <c r="E99" s="9"/>
-      <c r="F99" s="12">
+      <c r="F99" s="11">
         <f>IFERROR(VLOOKUP(E99, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1721,7 +1703,7 @@
       <c r="C100" s="10"/>
       <c r="D100" s="9"/>
       <c r="E100" s="9"/>
-      <c r="F100" s="12">
+      <c r="F100" s="11">
         <f>IFERROR(VLOOKUP(E100, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1734,7 +1716,7 @@
       <c r="C101" s="10"/>
       <c r="D101" s="9"/>
       <c r="E101" s="9"/>
-      <c r="F101" s="12">
+      <c r="F101" s="11">
         <f>IFERROR(VLOOKUP(E101, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1747,7 +1729,7 @@
       <c r="C102" s="10"/>
       <c r="D102" s="9"/>
       <c r="E102" s="9"/>
-      <c r="F102" s="12">
+      <c r="F102" s="11">
         <f>IFERROR(VLOOKUP(E102, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1760,7 +1742,7 @@
       <c r="C103" s="10"/>
       <c r="D103" s="9"/>
       <c r="E103" s="9"/>
-      <c r="F103" s="12">
+      <c r="F103" s="11">
         <f>IFERROR(VLOOKUP(E103, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1773,7 +1755,7 @@
       <c r="C104" s="10"/>
       <c r="D104" s="9"/>
       <c r="E104" s="9"/>
-      <c r="F104" s="12">
+      <c r="F104" s="11">
         <f>IFERROR(VLOOKUP(E104, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1786,13 +1768,13 @@
       <c r="C105" s="10"/>
       <c r="D105" s="9"/>
       <c r="E105" s="9"/>
-      <c r="F105" s="12">
+      <c r="F105" s="11">
         <f>IFERROR(VLOOKUP(E105, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="106" ht="15.75" customHeight="1">
-      <c r="A106" s="14"/>
+      <c r="A106" s="12"/>
     </row>
     <row r="107" ht="15.75" customHeight="1"/>
     <row r="108" ht="15.75" customHeight="1"/>
@@ -2694,15 +2676,22 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
   </mergeCells>
+  <conditionalFormatting sqref="C6:C105">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFFFFF"/>
+        <color rgb="FF57BB8A"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" showInputMessage="1" prompt="Digite uma data válida (DD/MM/AAAA" sqref="C6:C105">
-      <formula1>OR(NOT(ISERROR(DATEVALUE(C6))), AND(ISNUMBER(C6), LEFT(CELL("format", C6))="D"))</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Clique e digite um valor da lista de itens" sqref="E6:E105">
+      <formula1>"Normal,Participação,Isento,Serviço"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Mas,Fem"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Clique e digite um valor da lista de itens" sqref="E6:E105">
-      <formula1>"Normal,Participação,Isento,Serviço"</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>
@@ -2721,42 +2710,42 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="12" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="14">
+      <c r="B2" s="12">
         <v>200.0</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="15">
+      <c r="B3" s="12">
         <v>100.0</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="14">
+      <c r="B4" s="12">
         <v>130.0</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="12">
         <v>0.0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel file with new data
</commit_message>
<xml_diff>
--- a/public/xlsx/736067c4-bd56-4c2e-8e0e-6bd9cfa9f39c.xlsx
+++ b/public/xlsx/736067c4-bd56-4c2e-8e0e-6bd9cfa9f39c.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Página1" sheetId="1" r:id="rId4"/>
-    <sheet state="hidden" name="config" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="config" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>LISTA DE INSCRIÇÕES</t>
   </si>
@@ -78,6 +78,9 @@
     <t>Valor</t>
   </si>
   <si>
+    <t>Isento</t>
+  </si>
+  <si>
     <t>Tipo de inscrição</t>
   </si>
   <si>
@@ -88,9 +91,6 @@
   </si>
   <si>
     <t>Serviço</t>
-  </si>
-  <si>
-    <t>Isento</t>
   </si>
 </sst>
 </file>
@@ -176,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -201,6 +201,9 @@
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
@@ -480,9 +483,12 @@
       <c r="B6" s="9"/>
       <c r="C6" s="10"/>
       <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="11">
-        <f>IFERROR(VLOOKUP(E6, config!$A$2:$B$3, 2, FALSE), 0)</f>
+      <c r="E6" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="12">
+        <f>IFERROR(VLOOKUP(E6, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -494,7 +500,7 @@
       <c r="C7" s="10"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
-      <c r="F7" s="11">
+      <c r="F7" s="12">
         <f>IFERROR(VLOOKUP(E7, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -507,7 +513,7 @@
       <c r="C8" s="10"/>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
-      <c r="F8" s="11">
+      <c r="F8" s="12">
         <f>IFERROR(VLOOKUP(E8, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -520,7 +526,7 @@
       <c r="C9" s="10"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
-      <c r="F9" s="11">
+      <c r="F9" s="12">
         <f>IFERROR(VLOOKUP(E9, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -533,7 +539,7 @@
       <c r="C10" s="10"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
-      <c r="F10" s="11">
+      <c r="F10" s="12">
         <f>IFERROR(VLOOKUP(E10, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -546,7 +552,7 @@
       <c r="C11" s="10"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
-      <c r="F11" s="11">
+      <c r="F11" s="12">
         <f>IFERROR(VLOOKUP(E11, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -559,7 +565,7 @@
       <c r="C12" s="10"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
-      <c r="F12" s="11">
+      <c r="F12" s="12">
         <f>IFERROR(VLOOKUP(E12, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -572,7 +578,7 @@
       <c r="C13" s="10"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
-      <c r="F13" s="11">
+      <c r="F13" s="12">
         <f>IFERROR(VLOOKUP(E13, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -585,7 +591,7 @@
       <c r="C14" s="10"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
-      <c r="F14" s="11">
+      <c r="F14" s="12">
         <f>IFERROR(VLOOKUP(E14, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -598,7 +604,7 @@
       <c r="C15" s="10"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
-      <c r="F15" s="11">
+      <c r="F15" s="12">
         <f>IFERROR(VLOOKUP(E15, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -611,7 +617,7 @@
       <c r="C16" s="10"/>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
-      <c r="F16" s="11">
+      <c r="F16" s="12">
         <f>IFERROR(VLOOKUP(E16, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -624,7 +630,7 @@
       <c r="C17" s="10"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
-      <c r="F17" s="11">
+      <c r="F17" s="12">
         <f>IFERROR(VLOOKUP(E17, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -637,7 +643,7 @@
       <c r="C18" s="10"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
-      <c r="F18" s="11">
+      <c r="F18" s="12">
         <f>IFERROR(VLOOKUP(E18, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -650,7 +656,7 @@
       <c r="C19" s="10"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
-      <c r="F19" s="11">
+      <c r="F19" s="12">
         <f>IFERROR(VLOOKUP(E19, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -663,7 +669,7 @@
       <c r="C20" s="10"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
-      <c r="F20" s="11">
+      <c r="F20" s="12">
         <f>IFERROR(VLOOKUP(E20, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -676,7 +682,7 @@
       <c r="C21" s="10"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
-      <c r="F21" s="11">
+      <c r="F21" s="12">
         <f>IFERROR(VLOOKUP(E21, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -689,7 +695,7 @@
       <c r="C22" s="10"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
-      <c r="F22" s="11">
+      <c r="F22" s="12">
         <f>IFERROR(VLOOKUP(E22, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -702,7 +708,7 @@
       <c r="C23" s="10"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
-      <c r="F23" s="11">
+      <c r="F23" s="12">
         <f>IFERROR(VLOOKUP(E23, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -715,7 +721,7 @@
       <c r="C24" s="10"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
-      <c r="F24" s="11">
+      <c r="F24" s="12">
         <f>IFERROR(VLOOKUP(E24, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -728,7 +734,7 @@
       <c r="C25" s="10"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
-      <c r="F25" s="11">
+      <c r="F25" s="12">
         <f>IFERROR(VLOOKUP(E25, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -741,7 +747,7 @@
       <c r="C26" s="10"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
-      <c r="F26" s="11">
+      <c r="F26" s="12">
         <f>IFERROR(VLOOKUP(E26, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -754,7 +760,7 @@
       <c r="C27" s="10"/>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
-      <c r="F27" s="11">
+      <c r="F27" s="12">
         <f>IFERROR(VLOOKUP(E27, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -767,7 +773,7 @@
       <c r="C28" s="10"/>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
-      <c r="F28" s="11">
+      <c r="F28" s="12">
         <f>IFERROR(VLOOKUP(E28, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -780,7 +786,7 @@
       <c r="C29" s="10"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
-      <c r="F29" s="11">
+      <c r="F29" s="12">
         <f>IFERROR(VLOOKUP(E29, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -793,7 +799,7 @@
       <c r="C30" s="10"/>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
-      <c r="F30" s="11">
+      <c r="F30" s="12">
         <f>IFERROR(VLOOKUP(E30, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -806,7 +812,7 @@
       <c r="C31" s="10"/>
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
-      <c r="F31" s="11">
+      <c r="F31" s="12">
         <f>IFERROR(VLOOKUP(E31, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -819,7 +825,7 @@
       <c r="C32" s="10"/>
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
-      <c r="F32" s="11">
+      <c r="F32" s="12">
         <f>IFERROR(VLOOKUP(E32, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -832,7 +838,7 @@
       <c r="C33" s="10"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
-      <c r="F33" s="11">
+      <c r="F33" s="12">
         <f>IFERROR(VLOOKUP(E33, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -845,7 +851,7 @@
       <c r="C34" s="10"/>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
-      <c r="F34" s="11">
+      <c r="F34" s="12">
         <f>IFERROR(VLOOKUP(E34, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -858,7 +864,7 @@
       <c r="C35" s="10"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
-      <c r="F35" s="11">
+      <c r="F35" s="12">
         <f>IFERROR(VLOOKUP(E35, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -871,7 +877,7 @@
       <c r="C36" s="10"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
-      <c r="F36" s="11">
+      <c r="F36" s="12">
         <f>IFERROR(VLOOKUP(E36, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -884,7 +890,7 @@
       <c r="C37" s="10"/>
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
-      <c r="F37" s="11">
+      <c r="F37" s="12">
         <f>IFERROR(VLOOKUP(E37, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -897,7 +903,7 @@
       <c r="C38" s="10"/>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
-      <c r="F38" s="11">
+      <c r="F38" s="12">
         <f>IFERROR(VLOOKUP(E38, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -910,7 +916,7 @@
       <c r="C39" s="10"/>
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
-      <c r="F39" s="11">
+      <c r="F39" s="12">
         <f>IFERROR(VLOOKUP(E39, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -923,7 +929,7 @@
       <c r="C40" s="10"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
-      <c r="F40" s="11">
+      <c r="F40" s="12">
         <f>IFERROR(VLOOKUP(E40, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -936,7 +942,7 @@
       <c r="C41" s="10"/>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
-      <c r="F41" s="11">
+      <c r="F41" s="12">
         <f>IFERROR(VLOOKUP(E41, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -949,7 +955,7 @@
       <c r="C42" s="10"/>
       <c r="D42" s="9"/>
       <c r="E42" s="9"/>
-      <c r="F42" s="11">
+      <c r="F42" s="12">
         <f>IFERROR(VLOOKUP(E42, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -962,7 +968,7 @@
       <c r="C43" s="10"/>
       <c r="D43" s="9"/>
       <c r="E43" s="9"/>
-      <c r="F43" s="11">
+      <c r="F43" s="12">
         <f>IFERROR(VLOOKUP(E43, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -975,7 +981,7 @@
       <c r="C44" s="10"/>
       <c r="D44" s="9"/>
       <c r="E44" s="9"/>
-      <c r="F44" s="11">
+      <c r="F44" s="12">
         <f>IFERROR(VLOOKUP(E44, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -988,7 +994,7 @@
       <c r="C45" s="10"/>
       <c r="D45" s="9"/>
       <c r="E45" s="9"/>
-      <c r="F45" s="11">
+      <c r="F45" s="12">
         <f>IFERROR(VLOOKUP(E45, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1001,7 +1007,7 @@
       <c r="C46" s="10"/>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
-      <c r="F46" s="11">
+      <c r="F46" s="12">
         <f>IFERROR(VLOOKUP(E46, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1014,7 +1020,7 @@
       <c r="C47" s="10"/>
       <c r="D47" s="9"/>
       <c r="E47" s="9"/>
-      <c r="F47" s="11">
+      <c r="F47" s="12">
         <f>IFERROR(VLOOKUP(E47, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1027,7 +1033,7 @@
       <c r="C48" s="10"/>
       <c r="D48" s="9"/>
       <c r="E48" s="9"/>
-      <c r="F48" s="11">
+      <c r="F48" s="12">
         <f>IFERROR(VLOOKUP(E48, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1040,7 +1046,7 @@
       <c r="C49" s="10"/>
       <c r="D49" s="9"/>
       <c r="E49" s="9"/>
-      <c r="F49" s="11">
+      <c r="F49" s="12">
         <f>IFERROR(VLOOKUP(E49, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1053,7 +1059,7 @@
       <c r="C50" s="10"/>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
-      <c r="F50" s="11">
+      <c r="F50" s="12">
         <f>IFERROR(VLOOKUP(E50, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1066,7 +1072,7 @@
       <c r="C51" s="10"/>
       <c r="D51" s="9"/>
       <c r="E51" s="9"/>
-      <c r="F51" s="11">
+      <c r="F51" s="12">
         <f>IFERROR(VLOOKUP(E51, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1079,7 +1085,7 @@
       <c r="C52" s="10"/>
       <c r="D52" s="9"/>
       <c r="E52" s="9"/>
-      <c r="F52" s="11">
+      <c r="F52" s="12">
         <f>IFERROR(VLOOKUP(E52, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1092,7 +1098,7 @@
       <c r="C53" s="10"/>
       <c r="D53" s="9"/>
       <c r="E53" s="9"/>
-      <c r="F53" s="11">
+      <c r="F53" s="12">
         <f>IFERROR(VLOOKUP(E53, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1105,7 +1111,7 @@
       <c r="C54" s="10"/>
       <c r="D54" s="9"/>
       <c r="E54" s="9"/>
-      <c r="F54" s="11">
+      <c r="F54" s="12">
         <f>IFERROR(VLOOKUP(E54, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1118,7 +1124,7 @@
       <c r="C55" s="10"/>
       <c r="D55" s="9"/>
       <c r="E55" s="9"/>
-      <c r="F55" s="11">
+      <c r="F55" s="12">
         <f>IFERROR(VLOOKUP(E55, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1131,7 +1137,7 @@
       <c r="C56" s="10"/>
       <c r="D56" s="9"/>
       <c r="E56" s="9"/>
-      <c r="F56" s="11">
+      <c r="F56" s="12">
         <f>IFERROR(VLOOKUP(E56, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1144,7 +1150,7 @@
       <c r="C57" s="10"/>
       <c r="D57" s="9"/>
       <c r="E57" s="9"/>
-      <c r="F57" s="11">
+      <c r="F57" s="12">
         <f>IFERROR(VLOOKUP(E57, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1157,7 +1163,7 @@
       <c r="C58" s="10"/>
       <c r="D58" s="9"/>
       <c r="E58" s="9"/>
-      <c r="F58" s="11">
+      <c r="F58" s="12">
         <f>IFERROR(VLOOKUP(E58, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1170,7 +1176,7 @@
       <c r="C59" s="10"/>
       <c r="D59" s="9"/>
       <c r="E59" s="9"/>
-      <c r="F59" s="11">
+      <c r="F59" s="12">
         <f>IFERROR(VLOOKUP(E59, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1183,7 +1189,7 @@
       <c r="C60" s="10"/>
       <c r="D60" s="9"/>
       <c r="E60" s="9"/>
-      <c r="F60" s="11">
+      <c r="F60" s="12">
         <f>IFERROR(VLOOKUP(E60, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1196,7 +1202,7 @@
       <c r="C61" s="10"/>
       <c r="D61" s="9"/>
       <c r="E61" s="9"/>
-      <c r="F61" s="11">
+      <c r="F61" s="12">
         <f>IFERROR(VLOOKUP(E61, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1209,7 +1215,7 @@
       <c r="C62" s="10"/>
       <c r="D62" s="9"/>
       <c r="E62" s="9"/>
-      <c r="F62" s="11">
+      <c r="F62" s="12">
         <f>IFERROR(VLOOKUP(E62, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1222,7 +1228,7 @@
       <c r="C63" s="10"/>
       <c r="D63" s="9"/>
       <c r="E63" s="9"/>
-      <c r="F63" s="11">
+      <c r="F63" s="12">
         <f>IFERROR(VLOOKUP(E63, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1235,7 +1241,7 @@
       <c r="C64" s="10"/>
       <c r="D64" s="9"/>
       <c r="E64" s="9"/>
-      <c r="F64" s="11">
+      <c r="F64" s="12">
         <f>IFERROR(VLOOKUP(E64, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1248,7 +1254,7 @@
       <c r="C65" s="10"/>
       <c r="D65" s="9"/>
       <c r="E65" s="9"/>
-      <c r="F65" s="11">
+      <c r="F65" s="12">
         <f>IFERROR(VLOOKUP(E65, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1261,7 +1267,7 @@
       <c r="C66" s="10"/>
       <c r="D66" s="9"/>
       <c r="E66" s="9"/>
-      <c r="F66" s="11">
+      <c r="F66" s="12">
         <f>IFERROR(VLOOKUP(E66, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1274,7 +1280,7 @@
       <c r="C67" s="10"/>
       <c r="D67" s="9"/>
       <c r="E67" s="9"/>
-      <c r="F67" s="11">
+      <c r="F67" s="12">
         <f>IFERROR(VLOOKUP(E67, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1287,7 +1293,7 @@
       <c r="C68" s="10"/>
       <c r="D68" s="9"/>
       <c r="E68" s="9"/>
-      <c r="F68" s="11">
+      <c r="F68" s="12">
         <f>IFERROR(VLOOKUP(E68, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1300,7 +1306,7 @@
       <c r="C69" s="10"/>
       <c r="D69" s="9"/>
       <c r="E69" s="9"/>
-      <c r="F69" s="11">
+      <c r="F69" s="12">
         <f>IFERROR(VLOOKUP(E69, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1313,7 +1319,7 @@
       <c r="C70" s="10"/>
       <c r="D70" s="9"/>
       <c r="E70" s="9"/>
-      <c r="F70" s="11">
+      <c r="F70" s="12">
         <f>IFERROR(VLOOKUP(E70, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1326,7 +1332,7 @@
       <c r="C71" s="10"/>
       <c r="D71" s="9"/>
       <c r="E71" s="9"/>
-      <c r="F71" s="11">
+      <c r="F71" s="12">
         <f>IFERROR(VLOOKUP(E71, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1339,7 +1345,7 @@
       <c r="C72" s="10"/>
       <c r="D72" s="9"/>
       <c r="E72" s="9"/>
-      <c r="F72" s="11">
+      <c r="F72" s="12">
         <f>IFERROR(VLOOKUP(E72, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1352,7 +1358,7 @@
       <c r="C73" s="10"/>
       <c r="D73" s="9"/>
       <c r="E73" s="9"/>
-      <c r="F73" s="11">
+      <c r="F73" s="12">
         <f>IFERROR(VLOOKUP(E73, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1365,7 +1371,7 @@
       <c r="C74" s="10"/>
       <c r="D74" s="9"/>
       <c r="E74" s="9"/>
-      <c r="F74" s="11">
+      <c r="F74" s="12">
         <f>IFERROR(VLOOKUP(E74, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1378,7 +1384,7 @@
       <c r="C75" s="10"/>
       <c r="D75" s="9"/>
       <c r="E75" s="9"/>
-      <c r="F75" s="11">
+      <c r="F75" s="12">
         <f>IFERROR(VLOOKUP(E75, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1391,7 +1397,7 @@
       <c r="C76" s="10"/>
       <c r="D76" s="9"/>
       <c r="E76" s="9"/>
-      <c r="F76" s="11">
+      <c r="F76" s="12">
         <f>IFERROR(VLOOKUP(E76, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1404,7 +1410,7 @@
       <c r="C77" s="10"/>
       <c r="D77" s="9"/>
       <c r="E77" s="9"/>
-      <c r="F77" s="11">
+      <c r="F77" s="12">
         <f>IFERROR(VLOOKUP(E77, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1417,7 +1423,7 @@
       <c r="C78" s="10"/>
       <c r="D78" s="9"/>
       <c r="E78" s="9"/>
-      <c r="F78" s="11">
+      <c r="F78" s="12">
         <f>IFERROR(VLOOKUP(E78, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1430,7 +1436,7 @@
       <c r="C79" s="10"/>
       <c r="D79" s="9"/>
       <c r="E79" s="9"/>
-      <c r="F79" s="11">
+      <c r="F79" s="12">
         <f>IFERROR(VLOOKUP(E79, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1443,7 +1449,7 @@
       <c r="C80" s="10"/>
       <c r="D80" s="9"/>
       <c r="E80" s="9"/>
-      <c r="F80" s="11">
+      <c r="F80" s="12">
         <f>IFERROR(VLOOKUP(E80, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1456,7 +1462,7 @@
       <c r="C81" s="10"/>
       <c r="D81" s="9"/>
       <c r="E81" s="9"/>
-      <c r="F81" s="11">
+      <c r="F81" s="12">
         <f>IFERROR(VLOOKUP(E81, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1469,7 +1475,7 @@
       <c r="C82" s="10"/>
       <c r="D82" s="9"/>
       <c r="E82" s="9"/>
-      <c r="F82" s="11">
+      <c r="F82" s="12">
         <f>IFERROR(VLOOKUP(E82, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1482,7 +1488,7 @@
       <c r="C83" s="10"/>
       <c r="D83" s="9"/>
       <c r="E83" s="9"/>
-      <c r="F83" s="11">
+      <c r="F83" s="12">
         <f>IFERROR(VLOOKUP(E83, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1495,7 +1501,7 @@
       <c r="C84" s="10"/>
       <c r="D84" s="9"/>
       <c r="E84" s="9"/>
-      <c r="F84" s="11">
+      <c r="F84" s="12">
         <f>IFERROR(VLOOKUP(E84, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1508,7 +1514,7 @@
       <c r="C85" s="10"/>
       <c r="D85" s="9"/>
       <c r="E85" s="9"/>
-      <c r="F85" s="11">
+      <c r="F85" s="12">
         <f>IFERROR(VLOOKUP(E85, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1521,7 +1527,7 @@
       <c r="C86" s="10"/>
       <c r="D86" s="9"/>
       <c r="E86" s="9"/>
-      <c r="F86" s="11">
+      <c r="F86" s="12">
         <f>IFERROR(VLOOKUP(E86, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1534,7 +1540,7 @@
       <c r="C87" s="10"/>
       <c r="D87" s="9"/>
       <c r="E87" s="9"/>
-      <c r="F87" s="11">
+      <c r="F87" s="12">
         <f>IFERROR(VLOOKUP(E87, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1547,7 +1553,7 @@
       <c r="C88" s="10"/>
       <c r="D88" s="9"/>
       <c r="E88" s="9"/>
-      <c r="F88" s="11">
+      <c r="F88" s="12">
         <f>IFERROR(VLOOKUP(E88, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1560,7 +1566,7 @@
       <c r="C89" s="10"/>
       <c r="D89" s="9"/>
       <c r="E89" s="9"/>
-      <c r="F89" s="11">
+      <c r="F89" s="12">
         <f>IFERROR(VLOOKUP(E89, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1573,7 +1579,7 @@
       <c r="C90" s="10"/>
       <c r="D90" s="9"/>
       <c r="E90" s="9"/>
-      <c r="F90" s="11">
+      <c r="F90" s="12">
         <f>IFERROR(VLOOKUP(E90, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1586,7 +1592,7 @@
       <c r="C91" s="10"/>
       <c r="D91" s="9"/>
       <c r="E91" s="9"/>
-      <c r="F91" s="11">
+      <c r="F91" s="12">
         <f>IFERROR(VLOOKUP(E91, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1599,7 +1605,7 @@
       <c r="C92" s="10"/>
       <c r="D92" s="9"/>
       <c r="E92" s="9"/>
-      <c r="F92" s="11">
+      <c r="F92" s="12">
         <f>IFERROR(VLOOKUP(E92, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1612,7 +1618,7 @@
       <c r="C93" s="10"/>
       <c r="D93" s="9"/>
       <c r="E93" s="9"/>
-      <c r="F93" s="11">
+      <c r="F93" s="12">
         <f>IFERROR(VLOOKUP(E93, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1625,7 +1631,7 @@
       <c r="C94" s="10"/>
       <c r="D94" s="9"/>
       <c r="E94" s="9"/>
-      <c r="F94" s="11">
+      <c r="F94" s="12">
         <f>IFERROR(VLOOKUP(E94, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1638,7 +1644,7 @@
       <c r="C95" s="10"/>
       <c r="D95" s="9"/>
       <c r="E95" s="9"/>
-      <c r="F95" s="11">
+      <c r="F95" s="12">
         <f>IFERROR(VLOOKUP(E95, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1651,7 +1657,7 @@
       <c r="C96" s="10"/>
       <c r="D96" s="9"/>
       <c r="E96" s="9"/>
-      <c r="F96" s="11">
+      <c r="F96" s="12">
         <f>IFERROR(VLOOKUP(E96, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1664,7 +1670,7 @@
       <c r="C97" s="10"/>
       <c r="D97" s="9"/>
       <c r="E97" s="9"/>
-      <c r="F97" s="11">
+      <c r="F97" s="12">
         <f>IFERROR(VLOOKUP(E97, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1677,7 +1683,7 @@
       <c r="C98" s="10"/>
       <c r="D98" s="9"/>
       <c r="E98" s="9"/>
-      <c r="F98" s="11">
+      <c r="F98" s="12">
         <f>IFERROR(VLOOKUP(E98, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1690,7 +1696,7 @@
       <c r="C99" s="10"/>
       <c r="D99" s="9"/>
       <c r="E99" s="9"/>
-      <c r="F99" s="11">
+      <c r="F99" s="12">
         <f>IFERROR(VLOOKUP(E99, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1703,7 +1709,7 @@
       <c r="C100" s="10"/>
       <c r="D100" s="9"/>
       <c r="E100" s="9"/>
-      <c r="F100" s="11">
+      <c r="F100" s="12">
         <f>IFERROR(VLOOKUP(E100, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1716,7 +1722,7 @@
       <c r="C101" s="10"/>
       <c r="D101" s="9"/>
       <c r="E101" s="9"/>
-      <c r="F101" s="11">
+      <c r="F101" s="12">
         <f>IFERROR(VLOOKUP(E101, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1729,7 +1735,7 @@
       <c r="C102" s="10"/>
       <c r="D102" s="9"/>
       <c r="E102" s="9"/>
-      <c r="F102" s="11">
+      <c r="F102" s="12">
         <f>IFERROR(VLOOKUP(E102, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1742,7 +1748,7 @@
       <c r="C103" s="10"/>
       <c r="D103" s="9"/>
       <c r="E103" s="9"/>
-      <c r="F103" s="11">
+      <c r="F103" s="12">
         <f>IFERROR(VLOOKUP(E103, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1755,7 +1761,7 @@
       <c r="C104" s="10"/>
       <c r="D104" s="9"/>
       <c r="E104" s="9"/>
-      <c r="F104" s="11">
+      <c r="F104" s="12">
         <f>IFERROR(VLOOKUP(E104, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
@@ -1768,13 +1774,13 @@
       <c r="C105" s="10"/>
       <c r="D105" s="9"/>
       <c r="E105" s="9"/>
-      <c r="F105" s="11">
+      <c r="F105" s="12">
         <f>IFERROR(VLOOKUP(E105, config!$A$2:$B$3, 2, FALSE), 0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="106" ht="15.75" customHeight="1">
-      <c r="A106" s="12"/>
+      <c r="A106" s="13"/>
     </row>
     <row r="107" ht="15.75" customHeight="1"/>
     <row r="108" ht="15.75" customHeight="1"/>
@@ -2688,7 +2694,7 @@
   </conditionalFormatting>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Clique e digite um valor da lista de itens" sqref="E6:E105">
-      <formula1>"Normal,Participação,Isento,Serviço"</formula1>
+      <formula1>"Normal,Participação,Serviço,Isento"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6:D105">
       <formula1>"Mas,Fem"</formula1>
@@ -2710,42 +2716,42 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="A2" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="13">
+        <v>200.0</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="A3" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="13">
+        <v>100.0</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="13">
+        <v>130.0</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="12">
-        <v>200.0</v>
-      </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="12">
-        <v>100.0</v>
-      </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="12">
-        <v>130.0</v>
-      </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="12">
+      <c r="B5" s="13">
         <v>0.0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel file with revised data
</commit_message>
<xml_diff>
--- a/public/xlsx/736067c4-bd56-4c2e-8e0e-6bd9cfa9f39c.xlsx
+++ b/public/xlsx/736067c4-bd56-4c2e-8e0e-6bd9cfa9f39c.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Página1" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="config" sheetId="2" r:id="rId5"/>
+    <sheet state="hidden" name="config" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>LISTA DE INSCRIÇÕES</t>
   </si>
@@ -78,9 +78,6 @@
     <t>Valor</t>
   </si>
   <si>
-    <t>Isento</t>
-  </si>
-  <si>
     <t>Tipo de inscrição</t>
   </si>
   <si>
@@ -91,6 +88,9 @@
   </si>
   <si>
     <t>Serviço</t>
+  </si>
+  <si>
+    <t>Isento</t>
   </si>
 </sst>
 </file>
@@ -483,9 +483,7 @@
       <c r="B6" s="9"/>
       <c r="C6" s="10"/>
       <c r="D6" s="9"/>
-      <c r="E6" s="11" t="s">
-        <v>10</v>
-      </c>
+      <c r="E6" s="11"/>
       <c r="F6" s="12">
         <f>IFERROR(VLOOKUP(E6, config!$A$2:$B$5, 2, FALSE), 0)
 </f>
@@ -2717,7 +2715,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>9</v>
@@ -2725,7 +2723,7 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" s="13">
         <v>200.0</v>
@@ -2733,7 +2731,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="13">
         <v>100.0</v>
@@ -2741,7 +2739,7 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="13">
         <v>130.0</v>
@@ -2749,7 +2747,7 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="13" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B5" s="13">
         <v>0.0</v>

</xml_diff>

<commit_message>
chore: update xlsx file with new binary content
</commit_message>
<xml_diff>
--- a/public/xlsx/736067c4-bd56-4c2e-8e0e-6bd9cfa9f39c.xlsx
+++ b/public/xlsx/736067c4-bd56-4c2e-8e0e-6bd9cfa9f39c.xlsx
@@ -497,9 +497,10 @@
       <c r="B7" s="9"/>
       <c r="C7" s="10"/>
       <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
+      <c r="E7" s="11"/>
       <c r="F7" s="12">
-        <f>IFERROR(VLOOKUP(E7, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E7, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -510,9 +511,10 @@
       <c r="B8" s="9"/>
       <c r="C8" s="10"/>
       <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
+      <c r="E8" s="11"/>
       <c r="F8" s="12">
-        <f>IFERROR(VLOOKUP(E8, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E8, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -538,7 +540,8 @@
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="F10" s="12">
-        <f>IFERROR(VLOOKUP(E10, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E10, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -551,7 +554,8 @@
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="F11" s="12">
-        <f>IFERROR(VLOOKUP(E11, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E11, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -564,7 +568,8 @@
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="12">
-        <f>IFERROR(VLOOKUP(E12, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E12, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -577,7 +582,8 @@
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="F13" s="12">
-        <f>IFERROR(VLOOKUP(E13, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E13, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -590,7 +596,8 @@
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
       <c r="F14" s="12">
-        <f>IFERROR(VLOOKUP(E14, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E14, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -603,7 +610,8 @@
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
       <c r="F15" s="12">
-        <f>IFERROR(VLOOKUP(E15, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E15, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -616,7 +624,8 @@
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
       <c r="F16" s="12">
-        <f>IFERROR(VLOOKUP(E16, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E16, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -627,9 +636,10 @@
       <c r="B17" s="9"/>
       <c r="C17" s="10"/>
       <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
+      <c r="E17" s="11"/>
       <c r="F17" s="12">
-        <f>IFERROR(VLOOKUP(E17, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E17, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -642,7 +652,8 @@
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
       <c r="F18" s="12">
-        <f>IFERROR(VLOOKUP(E18, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E18, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -655,7 +666,8 @@
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="12">
-        <f>IFERROR(VLOOKUP(E19, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E19, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -666,9 +678,10 @@
       <c r="B20" s="9"/>
       <c r="C20" s="10"/>
       <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
+      <c r="E20" s="11"/>
       <c r="F20" s="12">
-        <f>IFERROR(VLOOKUP(E20, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E20, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -681,7 +694,8 @@
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="12">
-        <f>IFERROR(VLOOKUP(E21, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E21, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -694,7 +708,8 @@
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
       <c r="F22" s="12">
-        <f>IFERROR(VLOOKUP(E22, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E22, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -707,7 +722,8 @@
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
       <c r="F23" s="12">
-        <f>IFERROR(VLOOKUP(E23, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E23, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -720,7 +736,8 @@
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="12">
-        <f>IFERROR(VLOOKUP(E24, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E24, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -733,7 +750,8 @@
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
       <c r="F25" s="12">
-        <f>IFERROR(VLOOKUP(E25, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E25, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -746,7 +764,8 @@
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="12">
-        <f>IFERROR(VLOOKUP(E26, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E26, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -759,7 +778,8 @@
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
       <c r="F27" s="12">
-        <f>IFERROR(VLOOKUP(E27, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E27, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -772,7 +792,8 @@
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
       <c r="F28" s="12">
-        <f>IFERROR(VLOOKUP(E28, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E28, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -785,7 +806,8 @@
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
       <c r="F29" s="12">
-        <f>IFERROR(VLOOKUP(E29, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E29, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -798,7 +820,8 @@
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
       <c r="F30" s="12">
-        <f>IFERROR(VLOOKUP(E30, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E30, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -811,7 +834,8 @@
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
       <c r="F31" s="12">
-        <f>IFERROR(VLOOKUP(E31, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E31, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -824,7 +848,8 @@
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
       <c r="F32" s="12">
-        <f>IFERROR(VLOOKUP(E32, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E32, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -837,7 +862,8 @@
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
       <c r="F33" s="12">
-        <f>IFERROR(VLOOKUP(E33, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E33, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -848,9 +874,10 @@
       <c r="B34" s="9"/>
       <c r="C34" s="10"/>
       <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
+      <c r="E34" s="11"/>
       <c r="F34" s="12">
-        <f>IFERROR(VLOOKUP(E34, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E34, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -863,7 +890,8 @@
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
       <c r="F35" s="12">
-        <f>IFERROR(VLOOKUP(E35, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E35, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -876,7 +904,8 @@
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
       <c r="F36" s="12">
-        <f>IFERROR(VLOOKUP(E36, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E36, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -889,7 +918,8 @@
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
       <c r="F37" s="12">
-        <f>IFERROR(VLOOKUP(E37, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E37, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -902,7 +932,8 @@
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
       <c r="F38" s="12">
-        <f>IFERROR(VLOOKUP(E38, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E38, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -915,7 +946,8 @@
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
       <c r="F39" s="12">
-        <f>IFERROR(VLOOKUP(E39, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E39, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -928,7 +960,8 @@
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
       <c r="F40" s="12">
-        <f>IFERROR(VLOOKUP(E40, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E40, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -941,7 +974,8 @@
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
       <c r="F41" s="12">
-        <f>IFERROR(VLOOKUP(E41, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E41, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -954,7 +988,8 @@
       <c r="D42" s="9"/>
       <c r="E42" s="9"/>
       <c r="F42" s="12">
-        <f>IFERROR(VLOOKUP(E42, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E42, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -967,7 +1002,8 @@
       <c r="D43" s="9"/>
       <c r="E43" s="9"/>
       <c r="F43" s="12">
-        <f>IFERROR(VLOOKUP(E43, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E43, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -980,7 +1016,8 @@
       <c r="D44" s="9"/>
       <c r="E44" s="9"/>
       <c r="F44" s="12">
-        <f>IFERROR(VLOOKUP(E44, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E44, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -993,7 +1030,8 @@
       <c r="D45" s="9"/>
       <c r="E45" s="9"/>
       <c r="F45" s="12">
-        <f>IFERROR(VLOOKUP(E45, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E45, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1006,7 +1044,8 @@
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
       <c r="F46" s="12">
-        <f>IFERROR(VLOOKUP(E46, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E46, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1019,7 +1058,8 @@
       <c r="D47" s="9"/>
       <c r="E47" s="9"/>
       <c r="F47" s="12">
-        <f>IFERROR(VLOOKUP(E47, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E47, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1032,7 +1072,8 @@
       <c r="D48" s="9"/>
       <c r="E48" s="9"/>
       <c r="F48" s="12">
-        <f>IFERROR(VLOOKUP(E48, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E48, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1045,7 +1086,8 @@
       <c r="D49" s="9"/>
       <c r="E49" s="9"/>
       <c r="F49" s="12">
-        <f>IFERROR(VLOOKUP(E49, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E49, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1058,7 +1100,8 @@
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
       <c r="F50" s="12">
-        <f>IFERROR(VLOOKUP(E50, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E50, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1071,7 +1114,8 @@
       <c r="D51" s="9"/>
       <c r="E51" s="9"/>
       <c r="F51" s="12">
-        <f>IFERROR(VLOOKUP(E51, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E51, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1084,7 +1128,8 @@
       <c r="D52" s="9"/>
       <c r="E52" s="9"/>
       <c r="F52" s="12">
-        <f>IFERROR(VLOOKUP(E52, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E52, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1097,7 +1142,8 @@
       <c r="D53" s="9"/>
       <c r="E53" s="9"/>
       <c r="F53" s="12">
-        <f>IFERROR(VLOOKUP(E53, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E53, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1110,7 +1156,8 @@
       <c r="D54" s="9"/>
       <c r="E54" s="9"/>
       <c r="F54" s="12">
-        <f>IFERROR(VLOOKUP(E54, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E54, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1123,7 +1170,8 @@
       <c r="D55" s="9"/>
       <c r="E55" s="9"/>
       <c r="F55" s="12">
-        <f>IFERROR(VLOOKUP(E55, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E55, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1136,7 +1184,8 @@
       <c r="D56" s="9"/>
       <c r="E56" s="9"/>
       <c r="F56" s="12">
-        <f>IFERROR(VLOOKUP(E56, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E56, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1149,7 +1198,8 @@
       <c r="D57" s="9"/>
       <c r="E57" s="9"/>
       <c r="F57" s="12">
-        <f>IFERROR(VLOOKUP(E57, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E57, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1162,7 +1212,8 @@
       <c r="D58" s="9"/>
       <c r="E58" s="9"/>
       <c r="F58" s="12">
-        <f>IFERROR(VLOOKUP(E58, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E58, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1175,7 +1226,8 @@
       <c r="D59" s="9"/>
       <c r="E59" s="9"/>
       <c r="F59" s="12">
-        <f>IFERROR(VLOOKUP(E59, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E59, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1188,7 +1240,8 @@
       <c r="D60" s="9"/>
       <c r="E60" s="9"/>
       <c r="F60" s="12">
-        <f>IFERROR(VLOOKUP(E60, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E60, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1201,7 +1254,8 @@
       <c r="D61" s="9"/>
       <c r="E61" s="9"/>
       <c r="F61" s="12">
-        <f>IFERROR(VLOOKUP(E61, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E61, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1214,7 +1268,8 @@
       <c r="D62" s="9"/>
       <c r="E62" s="9"/>
       <c r="F62" s="12">
-        <f>IFERROR(VLOOKUP(E62, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E62, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1227,7 +1282,8 @@
       <c r="D63" s="9"/>
       <c r="E63" s="9"/>
       <c r="F63" s="12">
-        <f>IFERROR(VLOOKUP(E63, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E63, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1240,7 +1296,8 @@
       <c r="D64" s="9"/>
       <c r="E64" s="9"/>
       <c r="F64" s="12">
-        <f>IFERROR(VLOOKUP(E64, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E64, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1253,7 +1310,8 @@
       <c r="D65" s="9"/>
       <c r="E65" s="9"/>
       <c r="F65" s="12">
-        <f>IFERROR(VLOOKUP(E65, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E65, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1266,7 +1324,8 @@
       <c r="D66" s="9"/>
       <c r="E66" s="9"/>
       <c r="F66" s="12">
-        <f>IFERROR(VLOOKUP(E66, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E66, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1279,7 +1338,8 @@
       <c r="D67" s="9"/>
       <c r="E67" s="9"/>
       <c r="F67" s="12">
-        <f>IFERROR(VLOOKUP(E67, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E67, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1292,7 +1352,8 @@
       <c r="D68" s="9"/>
       <c r="E68" s="9"/>
       <c r="F68" s="12">
-        <f>IFERROR(VLOOKUP(E68, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E68, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1305,7 +1366,8 @@
       <c r="D69" s="9"/>
       <c r="E69" s="9"/>
       <c r="F69" s="12">
-        <f>IFERROR(VLOOKUP(E69, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E69, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1318,7 +1380,8 @@
       <c r="D70" s="9"/>
       <c r="E70" s="9"/>
       <c r="F70" s="12">
-        <f>IFERROR(VLOOKUP(E70, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E70, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1331,7 +1394,8 @@
       <c r="D71" s="9"/>
       <c r="E71" s="9"/>
       <c r="F71" s="12">
-        <f>IFERROR(VLOOKUP(E71, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E71, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1344,7 +1408,8 @@
       <c r="D72" s="9"/>
       <c r="E72" s="9"/>
       <c r="F72" s="12">
-        <f>IFERROR(VLOOKUP(E72, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E72, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1357,7 +1422,8 @@
       <c r="D73" s="9"/>
       <c r="E73" s="9"/>
       <c r="F73" s="12">
-        <f>IFERROR(VLOOKUP(E73, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E73, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1370,7 +1436,8 @@
       <c r="D74" s="9"/>
       <c r="E74" s="9"/>
       <c r="F74" s="12">
-        <f>IFERROR(VLOOKUP(E74, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E74, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1383,7 +1450,8 @@
       <c r="D75" s="9"/>
       <c r="E75" s="9"/>
       <c r="F75" s="12">
-        <f>IFERROR(VLOOKUP(E75, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E75, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1396,7 +1464,8 @@
       <c r="D76" s="9"/>
       <c r="E76" s="9"/>
       <c r="F76" s="12">
-        <f>IFERROR(VLOOKUP(E76, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E76, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1409,7 +1478,8 @@
       <c r="D77" s="9"/>
       <c r="E77" s="9"/>
       <c r="F77" s="12">
-        <f>IFERROR(VLOOKUP(E77, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E77, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1422,7 +1492,8 @@
       <c r="D78" s="9"/>
       <c r="E78" s="9"/>
       <c r="F78" s="12">
-        <f>IFERROR(VLOOKUP(E78, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E78, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1435,7 +1506,8 @@
       <c r="D79" s="9"/>
       <c r="E79" s="9"/>
       <c r="F79" s="12">
-        <f>IFERROR(VLOOKUP(E79, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E79, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1448,7 +1520,8 @@
       <c r="D80" s="9"/>
       <c r="E80" s="9"/>
       <c r="F80" s="12">
-        <f>IFERROR(VLOOKUP(E80, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E80, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1461,7 +1534,8 @@
       <c r="D81" s="9"/>
       <c r="E81" s="9"/>
       <c r="F81" s="12">
-        <f>IFERROR(VLOOKUP(E81, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E81, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1474,7 +1548,8 @@
       <c r="D82" s="9"/>
       <c r="E82" s="9"/>
       <c r="F82" s="12">
-        <f>IFERROR(VLOOKUP(E82, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E82, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1487,7 +1562,8 @@
       <c r="D83" s="9"/>
       <c r="E83" s="9"/>
       <c r="F83" s="12">
-        <f>IFERROR(VLOOKUP(E83, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E83, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1500,7 +1576,8 @@
       <c r="D84" s="9"/>
       <c r="E84" s="9"/>
       <c r="F84" s="12">
-        <f>IFERROR(VLOOKUP(E84, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E84, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1513,7 +1590,8 @@
       <c r="D85" s="9"/>
       <c r="E85" s="9"/>
       <c r="F85" s="12">
-        <f>IFERROR(VLOOKUP(E85, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E85, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1526,7 +1604,8 @@
       <c r="D86" s="9"/>
       <c r="E86" s="9"/>
       <c r="F86" s="12">
-        <f>IFERROR(VLOOKUP(E86, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E86, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1539,7 +1618,8 @@
       <c r="D87" s="9"/>
       <c r="E87" s="9"/>
       <c r="F87" s="12">
-        <f>IFERROR(VLOOKUP(E87, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E87, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1552,7 +1632,8 @@
       <c r="D88" s="9"/>
       <c r="E88" s="9"/>
       <c r="F88" s="12">
-        <f>IFERROR(VLOOKUP(E88, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E88, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1565,7 +1646,8 @@
       <c r="D89" s="9"/>
       <c r="E89" s="9"/>
       <c r="F89" s="12">
-        <f>IFERROR(VLOOKUP(E89, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E89, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1578,7 +1660,8 @@
       <c r="D90" s="9"/>
       <c r="E90" s="9"/>
       <c r="F90" s="12">
-        <f>IFERROR(VLOOKUP(E90, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E90, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1591,7 +1674,8 @@
       <c r="D91" s="9"/>
       <c r="E91" s="9"/>
       <c r="F91" s="12">
-        <f>IFERROR(VLOOKUP(E91, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E91, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1604,7 +1688,8 @@
       <c r="D92" s="9"/>
       <c r="E92" s="9"/>
       <c r="F92" s="12">
-        <f>IFERROR(VLOOKUP(E92, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E92, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1617,7 +1702,8 @@
       <c r="D93" s="9"/>
       <c r="E93" s="9"/>
       <c r="F93" s="12">
-        <f>IFERROR(VLOOKUP(E93, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E93, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1630,7 +1716,8 @@
       <c r="D94" s="9"/>
       <c r="E94" s="9"/>
       <c r="F94" s="12">
-        <f>IFERROR(VLOOKUP(E94, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E94, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1643,7 +1730,8 @@
       <c r="D95" s="9"/>
       <c r="E95" s="9"/>
       <c r="F95" s="12">
-        <f>IFERROR(VLOOKUP(E95, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E95, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1656,7 +1744,8 @@
       <c r="D96" s="9"/>
       <c r="E96" s="9"/>
       <c r="F96" s="12">
-        <f>IFERROR(VLOOKUP(E96, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E96, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1669,7 +1758,8 @@
       <c r="D97" s="9"/>
       <c r="E97" s="9"/>
       <c r="F97" s="12">
-        <f>IFERROR(VLOOKUP(E97, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E97, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1682,7 +1772,8 @@
       <c r="D98" s="9"/>
       <c r="E98" s="9"/>
       <c r="F98" s="12">
-        <f>IFERROR(VLOOKUP(E98, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E98, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1695,7 +1786,8 @@
       <c r="D99" s="9"/>
       <c r="E99" s="9"/>
       <c r="F99" s="12">
-        <f>IFERROR(VLOOKUP(E99, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E99, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1708,7 +1800,8 @@
       <c r="D100" s="9"/>
       <c r="E100" s="9"/>
       <c r="F100" s="12">
-        <f>IFERROR(VLOOKUP(E100, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E100, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1721,7 +1814,8 @@
       <c r="D101" s="9"/>
       <c r="E101" s="9"/>
       <c r="F101" s="12">
-        <f>IFERROR(VLOOKUP(E101, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E101, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1734,7 +1828,8 @@
       <c r="D102" s="9"/>
       <c r="E102" s="9"/>
       <c r="F102" s="12">
-        <f>IFERROR(VLOOKUP(E102, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E102, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1747,7 +1842,8 @@
       <c r="D103" s="9"/>
       <c r="E103" s="9"/>
       <c r="F103" s="12">
-        <f>IFERROR(VLOOKUP(E103, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E103, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1760,7 +1856,8 @@
       <c r="D104" s="9"/>
       <c r="E104" s="9"/>
       <c r="F104" s="12">
-        <f>IFERROR(VLOOKUP(E104, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E104, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>
@@ -1773,7 +1870,8 @@
       <c r="D105" s="9"/>
       <c r="E105" s="9"/>
       <c r="F105" s="12">
-        <f>IFERROR(VLOOKUP(E105, config!$A$2:$B$3, 2, FALSE), 0)</f>
+        <f>IFERROR(VLOOKUP(E105, config!$A$2:$B$5, 2, FALSE), 0)
+</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>